<commit_message>
refactor(core): fully deprecate redundant doctorCode in favor of UID across DB, API, and UI
</commit_message>
<xml_diff>
--- a/REPORTING MODULE/Stockist List-Alfez.xlsx
+++ b/REPORTING MODULE/Stockist List-Alfez.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MY WORK FLOW\Emyris Onboard App\REPORTING MODULE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CF6A9B1-9181-472A-9F31-1C4FC10A4EE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BC9FC47-C410-480A-83E1-F284EDC2F7B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,10 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="32">
-  <si>
-    <t>Sr</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="29">
   <si>
     <t>Business Name</t>
   </si>
@@ -55,12 +52,6 @@
   </si>
   <si>
     <t>City</t>
-  </si>
-  <si>
-    <t>Working Area</t>
-  </si>
-  <si>
-    <t>UID</t>
   </si>
   <si>
     <t>devraj parmar</t>
@@ -499,27 +490,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.75" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.25" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="142.625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.25" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="142.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>31</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -545,172 +535,139 @@
       <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" t="s">
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>9</v>
       </c>
-      <c r="L1" t="s">
+      <c r="B2" t="s">
         <v>10</v>
       </c>
-      <c r="M1" t="s">
-        <v>11</v>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J2" t="s">
+        <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" t="s">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" t="s">
+        <v>11</v>
+      </c>
+      <c r="H3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J3" t="s">
         <v>14</v>
       </c>
-      <c r="E2" t="s">
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4" t="s">
         <v>14</v>
       </c>
-      <c r="F2" t="s">
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I5" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5" t="s">
         <v>14</v>
-      </c>
-      <c r="G2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2" t="s">
-        <v>15</v>
-      </c>
-      <c r="J2" t="s">
-        <v>16</v>
-      </c>
-      <c r="K2" t="s">
-        <v>17</v>
-      </c>
-      <c r="L2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I3" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3" t="s">
-        <v>21</v>
-      </c>
-      <c r="K3" t="s">
-        <v>17</v>
-      </c>
-      <c r="L3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" t="s">
-        <v>14</v>
-      </c>
-      <c r="I4" t="s">
-        <v>25</v>
-      </c>
-      <c r="J4" t="s">
-        <v>26</v>
-      </c>
-      <c r="K4" t="s">
-        <v>17</v>
-      </c>
-      <c r="L4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" t="s">
-        <v>14</v>
-      </c>
-      <c r="G5" t="s">
-        <v>14</v>
-      </c>
-      <c r="H5" t="s">
-        <v>14</v>
-      </c>
-      <c r="I5" t="s">
-        <v>29</v>
-      </c>
-      <c r="J5" t="s">
-        <v>30</v>
-      </c>
-      <c r="K5" t="s">
-        <v>17</v>
-      </c>
-      <c r="L5" t="s">
-        <v>17</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1 A6:M6 A2:L5 D7:M8 C1:M1" numberStoredAsText="1"/>
+    <ignoredError sqref="A6:J6 A2:J5 B1:J1 C7:J8" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>